<commit_message>
added logic to handle uat landing page
</commit_message>
<xml_diff>
--- a/src/test/resources/TestCoverageDashboard_UAT.xlsx
+++ b/src/test/resources/TestCoverageDashboard_UAT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\57901\smart-test-automation\src\test\resources\"/>
     </mc:Choice>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
   <si>
     <t>Functional Area</t>
   </si>
@@ -158,6 +158,12 @@
   </si>
   <si>
     <t>03/30/2026 05:50:29 PM</t>
+  </si>
+  <si>
+    <t>04/14/2026 06:36:12 PM</t>
+  </si>
+  <si>
+    <t>04/14/2026 07:55:21 PM</t>
   </si>
 </sst>
 </file>
@@ -3455,14 +3461,14 @@
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" customWidth="1"/>
-    <col min="2" max="3" width="24.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" customWidth="1"/>
-    <col min="6" max="6" width="8.140625" customWidth="1"/>
-    <col min="7" max="7" width="7.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="34.7109375"/>
+    <col min="2" max="3" customWidth="true" width="24.5703125"/>
+    <col min="4" max="4" customWidth="true" width="14.7109375"/>
+    <col min="5" max="5" customWidth="true" width="9.140625"/>
+    <col min="6" max="6" customWidth="true" width="8.140625"/>
+    <col min="7" max="7" customWidth="true" width="7.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.28515625"/>
+    <col min="9" max="9" customWidth="true" width="24.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3470,7 +3476,7 @@
         <v>26</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C1" s="26">
         <v>46111.738459328706</v>
@@ -3511,29 +3517,29 @@
       <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="9">
-        <v>31</v>
-      </c>
-      <c r="C3" s="9">
-        <v>29</v>
-      </c>
-      <c r="D3" s="9">
-        <v>2</v>
-      </c>
-      <c r="E3" s="9">
-        <v>0</v>
-      </c>
-      <c r="F3" s="7">
+      <c r="B3" s="9" t="n">
+        <v>31.0</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>29.0</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="7" t="n">
         <f>IF(B3=0,"",C3/B3)</f>
-        <v>0.93548387096774188</v>
-      </c>
-      <c r="G3" s="7">
+        <v>0.9354838709677419</v>
+      </c>
+      <c r="G3" s="7" t="n">
         <f>IFERROR(D3/B3,0)</f>
-        <v>6.4516129032258063E-2</v>
-      </c>
-      <c r="H3" s="7">
+        <v>0.06451612903225806</v>
+      </c>
+      <c r="H3" s="7" t="n">
         <f>IFERROR(E3/B3,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
@@ -3552,162 +3558,162 @@
       <c r="E4" s="10">
         <v>0</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="7" t="n">
         <f t="shared" ref="F4:F16" si="0">IF(B4=0,"",C4/B4)</f>
-        <v>1</v>
-      </c>
-      <c r="G4" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G4" s="7" t="n">
         <f t="shared" ref="G4:G14" si="1">IFERROR(D4/B4,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H4" s="7" t="n">
         <f t="shared" ref="H4:H14" si="2">IFERROR(E4/B4,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="9">
-        <v>9</v>
-      </c>
-      <c r="C5" s="9">
-        <v>9</v>
-      </c>
-      <c r="D5" s="9">
-        <v>0</v>
-      </c>
-      <c r="E5" s="9">
-        <v>0</v>
-      </c>
-      <c r="F5" s="7">
+      <c r="B5" s="9" t="n">
+        <v>9.0</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F5" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G5" s="7">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G5" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H5" s="7">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="H5" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="10">
-        <v>7</v>
-      </c>
-      <c r="C6" s="10">
-        <v>7</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0</v>
-      </c>
-      <c r="E6" s="10">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7">
+      <c r="B6" s="10" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G6" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G6" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H6" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="9">
-        <v>17</v>
-      </c>
-      <c r="C7" s="9">
-        <v>17</v>
-      </c>
-      <c r="D7" s="9">
-        <v>0</v>
-      </c>
-      <c r="E7" s="9">
-        <v>0</v>
-      </c>
-      <c r="F7" s="7">
+      <c r="B7" s="9" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G7" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G7" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H7" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H7" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="9">
-        <v>7</v>
-      </c>
-      <c r="C8" s="10">
-        <v>7</v>
-      </c>
-      <c r="D8" s="10">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10">
-        <v>0</v>
-      </c>
-      <c r="F8" s="7">
+      <c r="B8" s="9" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G8" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G8" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H8" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H8" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="9">
-        <v>8</v>
-      </c>
-      <c r="C9" s="9">
-        <v>8</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="9">
-        <v>0</v>
-      </c>
-      <c r="F9" s="7">
+      <c r="B9" s="9" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G9" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G9" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -3723,13 +3729,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H10" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H10" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I10" s="2"/>
     </row>
@@ -3745,13 +3751,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H11" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I11" s="2"/>
     </row>
@@ -3767,13 +3773,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H12" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I12" s="2"/>
     </row>
@@ -3781,29 +3787,29 @@
       <c r="A13" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="9">
-        <v>1</v>
-      </c>
-      <c r="C13" s="9">
-        <v>0</v>
-      </c>
-      <c r="D13" s="9">
-        <v>1</v>
-      </c>
-      <c r="E13" s="9">
-        <v>0</v>
-      </c>
-      <c r="F13" s="7">
+      <c r="B13" s="9" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F13" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="7">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="G13" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="H13" s="7">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="H13" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -3819,13 +3825,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H14" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -3833,29 +3839,29 @@
       <c r="A15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="9">
-        <v>10</v>
-      </c>
-      <c r="C15" s="9">
-        <v>10</v>
-      </c>
-      <c r="D15" s="9">
-        <v>0</v>
-      </c>
-      <c r="E15" s="9">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7">
+      <c r="B15" s="9" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G15" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <f>IFERROR(D15/B15,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <f t="shared" ref="H15:H17" si="3">IFERROR(E15/B15,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
@@ -3870,46 +3876,46 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="7" t="n">
         <f>IFERROR(D16/B16,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H16" s="7" t="n">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="14" t="n">
         <f>SUM(B3:B16)</f>
-        <v>98</v>
-      </c>
-      <c r="C17" s="14">
+        <v>104.0</v>
+      </c>
+      <c r="C17" s="14" t="n">
         <f>SUM(C3:C15)</f>
-        <v>95</v>
-      </c>
-      <c r="D17" s="14">
+        <v>99.0</v>
+      </c>
+      <c r="D17" s="14" t="n">
         <f>SUM(D3:D15)</f>
-        <v>3</v>
-      </c>
-      <c r="E17" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="E17" s="14" t="n">
         <f>SUM(E3:E15)</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="15">
+        <v>0.0</v>
+      </c>
+      <c r="F17" s="15" t="n">
         <f t="shared" ref="F17" si="4">IFERROR(C17/B17,0)</f>
-        <v>0.96938775510204078</v>
-      </c>
-      <c r="G17" s="15">
+        <v>0.9519230769230769</v>
+      </c>
+      <c r="G17" s="15" t="n">
         <f t="shared" ref="G17" si="5">IFERROR(D17/B17,0)</f>
-        <v>3.0612244897959183E-2</v>
-      </c>
-      <c r="H17" s="15">
+        <v>0.04807692307692308</v>
+      </c>
+      <c r="H17" s="15" t="n">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>
@@ -3954,12 +3960,12 @@
   <dimension ref="A1:P8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="25.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="8" max="8" width="49.140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="14.7109375"/>
+    <col min="2" max="2" customWidth="true" width="23.5703125"/>
+    <col min="5" max="5" customWidth="true" width="18.0"/>
+    <col min="6" max="6" customWidth="true" width="25.7109375"/>
+    <col min="7" max="7" customWidth="true" width="15.85546875"/>
+    <col min="8" max="8" customWidth="true" width="49.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="33" x14ac:dyDescent="0.25">
@@ -3988,7 +3994,7 @@
       </c>
       <c r="H3" s="5" t="str">
         <f>TestCoverage!B1</f>
-        <v>03/30/2026 05:50:29 PM</v>
+        <v>04/14/2026 07:55:21 PM</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -4003,9 +4009,9 @@
       <c r="G4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="17">
+      <c r="H4" s="17" t="n">
         <f>TestCoverage!B17</f>
-        <v>98</v>
+        <v>104.0</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
@@ -4020,9 +4026,9 @@
       <c r="G5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="17" t="n">
         <f>TestCoverage!C17</f>
-        <v>95</v>
+        <v>99.0</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -4037,9 +4043,9 @@
       <c r="G6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="17">
+      <c r="H6" s="17" t="n">
         <f>TestCoverage!D17</f>
-        <v>3</v>
+        <v>5.0</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -4054,9 +4060,9 @@
       <c r="G7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="17" t="n">
         <f>TestCoverage!E17</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -4071,9 +4077,9 @@
       <c r="G8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="16">
+      <c r="H8" s="16" t="n">
         <f>IFERROR(H5/H4,"")</f>
-        <v>0.96938775510204078</v>
+        <v>0.9519230769230769</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -4123,14 +4129,14 @@
   <dimension ref="A1:J16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="4" max="5" width="13.85546875" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" customWidth="1"/>
-    <col min="7" max="7" width="26.140625" customWidth="1"/>
-    <col min="8" max="8" width="23.5703125" customWidth="1"/>
-    <col min="9" max="9" width="39.140625" customWidth="1"/>
-    <col min="10" max="10" width="33.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="37.85546875"/>
+    <col min="2" max="2" customWidth="true" width="14.0"/>
+    <col min="4" max="5" customWidth="true" width="13.85546875"/>
+    <col min="6" max="6" customWidth="true" width="10.42578125"/>
+    <col min="7" max="7" customWidth="true" width="26.140625"/>
+    <col min="8" max="8" customWidth="true" width="23.5703125"/>
+    <col min="9" max="9" customWidth="true" width="39.140625"/>
+    <col min="10" max="10" customWidth="true" width="33.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -4158,7 +4164,7 @@
       <c r="H1" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>34</v>
       </c>
       <c r="J1" s="24" t="s">
@@ -4168,31 +4174,31 @@
     <row r="2" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="str">
         <f>TestCoverage!A13 &amp; " (" &amp; IFERROR(TestCoverage!B13+0,0) &amp; ")"</f>
-        <v>Accessibility (Section 508 Compliance) (1)</v>
-      </c>
-      <c r="B2" s="20">
+        <v>Accessibility (Section 508 Compliance) (7)</v>
+      </c>
+      <c r="B2" s="20" t="n">
         <f>TestCoverage!F13</f>
-        <v>0</v>
-      </c>
-      <c r="C2" s="20">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="C2" s="20" t="n">
         <f>TestCoverage!G13</f>
-        <v>1</v>
-      </c>
-      <c r="D2" s="20">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="D2" s="20" t="n">
         <f>TestCoverage!H13</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="20" t="n">
         <f>C2 + D2</f>
-        <v>1</v>
-      </c>
-      <c r="F2" s="19">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="F2" s="19" t="n">
         <f>TestCoverage!B13</f>
-        <v>1</v>
-      </c>
-      <c r="G2" s="18">
+        <v>7.0</v>
+      </c>
+      <c r="G2" s="18" t="n">
         <f>IF($F2=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H2" s="19" t="str">
         <f>IF(G2=100%,"Not Automated","")</f>
@@ -4200,7 +4206,7 @@
       </c>
       <c r="I2" s="19" t="str">
         <f>IF(AND(C2&gt;0,F2&gt;0),"⚠️ "&amp;A2,A2)</f>
-        <v>⚠️ Accessibility (Section 508 Compliance) (1)</v>
+        <v>⚠️ Accessibility (Section 508 Compliance) (7)</v>
       </c>
       <c r="J2" s="19" t="str">
         <f>IF(D2=100%,"Blocked","")</f>
@@ -4212,29 +4218,29 @@
         <f>TestCoverage!A3 &amp; " (" &amp; IFERROR(TestCoverage!B3+0,0) &amp; ")"</f>
         <v>Validations &amp; Business Rules (31)</v>
       </c>
-      <c r="B3" s="20">
+      <c r="B3" s="20" t="n">
         <f>TestCoverage!F3</f>
-        <v>0.93548387096774188</v>
-      </c>
-      <c r="C3" s="20">
+        <v>0.9354838709677419</v>
+      </c>
+      <c r="C3" s="20" t="n">
         <f>TestCoverage!G3</f>
-        <v>6.4516129032258063E-2</v>
-      </c>
-      <c r="D3" s="20">
+        <v>0.06451612903225806</v>
+      </c>
+      <c r="D3" s="20" t="n">
         <f>TestCoverage!H3</f>
-        <v>0</v>
-      </c>
-      <c r="E3" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E3" s="20" t="n">
         <f>C3 + D3</f>
-        <v>6.4516129032258063E-2</v>
-      </c>
-      <c r="F3" s="19">
+        <v>0.06451612903225806</v>
+      </c>
+      <c r="F3" s="19" t="n">
         <f>TestCoverage!B3</f>
-        <v>31</v>
-      </c>
-      <c r="G3" s="18">
+        <v>31.0</v>
+      </c>
+      <c r="G3" s="18" t="n">
         <f>IF($F3=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H3" s="19" t="str">
         <f>IF(G3=100%,"Not Automated","")</f>
@@ -4254,29 +4260,29 @@
         <f>TestCoverage!A4 &amp; " (" &amp; IFERROR(TestCoverage!B4+0,0) &amp; ")"</f>
         <v>RAI Management (8)</v>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="20" t="n">
         <f>TestCoverage!F4</f>
-        <v>1</v>
-      </c>
-      <c r="C4" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="C4" s="20" t="n">
         <f>TestCoverage!G4</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D4" s="20" t="n">
         <f>TestCoverage!H4</f>
-        <v>0</v>
-      </c>
-      <c r="E4" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="20" t="n">
         <f>C4 + D4</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="19" t="n">
         <f>TestCoverage!B4</f>
-        <v>8</v>
-      </c>
-      <c r="G4" s="18">
+        <v>8.0</v>
+      </c>
+      <c r="G4" s="18" t="n">
         <f>IF($F4=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H4" s="19" t="str">
         <f>IF(G4=100%,"Not Automated","")</f>
@@ -4296,29 +4302,29 @@
         <f>TestCoverage!A5 &amp; " (" &amp; IFERROR(TestCoverage!B5+0,0) &amp; ")"</f>
         <v>SRT Review (9)</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="20" t="n">
         <f>TestCoverage!F5</f>
-        <v>1</v>
-      </c>
-      <c r="C5" s="20">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="C5" s="20" t="n">
         <f>TestCoverage!G5</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="20">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="D5" s="20" t="n">
         <f>TestCoverage!H5</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E5" s="20" t="n">
         <f>C5 + D5</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="19">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="F5" s="19" t="n">
         <f>TestCoverage!B5</f>
-        <v>9</v>
-      </c>
-      <c r="G5" s="18">
+        <v>9.0</v>
+      </c>
+      <c r="G5" s="18" t="n">
         <f>IF($F5=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H5" s="19" t="str">
         <f>IF(G5=100%,"Not Automated","")</f>
@@ -4326,7 +4332,7 @@
       </c>
       <c r="I5" s="19" t="str">
         <f>IF(AND(C5&gt;0,F5&gt;0),"⚠️ "&amp;A5,A5)</f>
-        <v>SRT Review (9)</v>
+        <v>⚠️ SRT Review (9)</v>
       </c>
       <c r="J5" s="19" t="str">
         <f>IF(D5=100%,"Blocked","")</f>
@@ -4338,29 +4344,29 @@
         <f>TestCoverage!A6 &amp; " (" &amp; IFERROR(TestCoverage!B6+0,0) &amp; ")"</f>
         <v>Workflow &amp; Status Transitions (7)</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="20" t="n">
         <f>TestCoverage!F6</f>
-        <v>1</v>
-      </c>
-      <c r="C6" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="C6" s="20" t="n">
         <f>TestCoverage!G6</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D6" s="20" t="n">
         <f>TestCoverage!H6</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="20" t="n">
         <f>C6 + D6</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="19" t="n">
         <f>TestCoverage!B6</f>
-        <v>7</v>
-      </c>
-      <c r="G6" s="18">
+        <v>7.0</v>
+      </c>
+      <c r="G6" s="18" t="n">
         <f>IF($F6=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H6" s="19" t="str">
         <f>IF(G6=100%,"Not Automated","")</f>
@@ -4380,29 +4386,29 @@
         <f>TestCoverage!A7 &amp; " (" &amp; IFERROR(TestCoverage!B7+0,0) &amp; ")"</f>
         <v>Record Lifecycle Management (17)</v>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="20" t="n">
         <f>TestCoverage!F7</f>
-        <v>1</v>
-      </c>
-      <c r="C7" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="C7" s="20" t="n">
         <f>TestCoverage!G7</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D7" s="20" t="n">
         <f>TestCoverage!H7</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E7" s="20" t="n">
         <f>C7 + D7</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="19" t="n">
         <f>TestCoverage!B7</f>
-        <v>17</v>
-      </c>
-      <c r="G7" s="18">
+        <v>17.0</v>
+      </c>
+      <c r="G7" s="18" t="n">
         <f>IF($F7=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H7" s="19" t="str">
         <f>IF(G7=100%,"Not Automated","")</f>
@@ -4422,29 +4428,29 @@
         <f>TestCoverage!A8 &amp; " (" &amp; IFERROR(TestCoverage!B8+0,0) &amp; ")"</f>
         <v>User Access &amp; Permissions (7)</v>
       </c>
-      <c r="B8" s="20">
+      <c r="B8" s="20" t="n">
         <f>TestCoverage!F8</f>
-        <v>1</v>
-      </c>
-      <c r="C8" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="C8" s="20" t="n">
         <f>TestCoverage!G8</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="20" t="n">
         <f>TestCoverage!H8</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="20" t="n">
         <f>C8 + D8</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="19" t="n">
         <f>TestCoverage!B8</f>
-        <v>7</v>
-      </c>
-      <c r="G8" s="18">
+        <v>7.0</v>
+      </c>
+      <c r="G8" s="18" t="n">
         <f>IF($F8=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H8" s="19" t="str">
         <f>IF(G8=100%,"Not Automated","")</f>
@@ -4464,29 +4470,29 @@
         <f>TestCoverage!A9 &amp; " (" &amp; IFERROR(TestCoverage!B9+0,0) &amp; ")"</f>
         <v>Assignment &amp; Routing (8)</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="20" t="n">
         <f>TestCoverage!F9</f>
-        <v>1</v>
-      </c>
-      <c r="C9" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="C9" s="20" t="n">
         <f>TestCoverage!G9</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="20" t="n">
         <f>TestCoverage!H9</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E9" s="20" t="n">
         <f>C9 + D9</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="19" t="n">
         <f>TestCoverage!B9</f>
-        <v>8</v>
-      </c>
-      <c r="G9" s="18">
+        <v>8.0</v>
+      </c>
+      <c r="G9" s="18" t="n">
         <f>IF($F9=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H9" s="19" t="str">
         <f>IF(G9=100%,"Not Automated","")</f>
@@ -4510,25 +4516,25 @@
         <f>TestCoverage!F10</f>
         <v/>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="20" t="n">
         <f>TestCoverage!G10</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D10" s="20" t="n">
         <f>TestCoverage!H10</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <f>C10 + D10</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F10" s="19" t="n">
         <f>TestCoverage!B10</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="18">
+        <v>0.0</v>
+      </c>
+      <c r="G10" s="18" t="n">
         <f>IF($F10=0,1,0)</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
       <c r="H10" s="19" t="str">
         <f>IF(G10=100%,"Not Automated","")</f>
@@ -4552,25 +4558,25 @@
         <f>TestCoverage!F11</f>
         <v/>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="20" t="n">
         <f>TestCoverage!G11</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="20" t="n">
         <f>TestCoverage!H11</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <f>C11 + D11</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F11" s="19" t="n">
         <f>TestCoverage!B11</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="18">
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="18" t="n">
         <f>IF($F11=0,1,0)</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
       <c r="H11" s="19" t="str">
         <f>IF(G11=100%,"Not Automated","")</f>
@@ -4594,25 +4600,25 @@
         <f>TestCoverage!F12</f>
         <v/>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="20" t="n">
         <f>TestCoverage!G12</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="20" t="n">
         <f>TestCoverage!H12</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <f>C12 + D12</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F12" s="19" t="n">
         <f>TestCoverage!B12</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="18">
+        <v>0.0</v>
+      </c>
+      <c r="G12" s="18" t="n">
         <f>IF($F12=0,1,0)</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
       <c r="H12" s="19" t="str">
         <f>IF(G12=100%,"Not Automated","")</f>
@@ -4636,25 +4642,25 @@
         <f>TestCoverage!F14</f>
         <v/>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="20" t="n">
         <f>TestCoverage!G14</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D13" s="20" t="n">
         <f>TestCoverage!H14</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E13" s="20" t="n">
         <f>C13 + D13</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F13" s="19" t="n">
         <f>TestCoverage!B14</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="18">
+        <v>0.0</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <f>IF($F13=0,1,0)</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
       <c r="H13" s="19" t="str">
         <f>IF(G13=100%,"Not Automated","")</f>
@@ -4674,29 +4680,29 @@
         <f>TestCoverage!A15 &amp; " (" &amp; IFERROR(TestCoverage!B15+0,0) &amp; ")"</f>
         <v>Timeline &amp; SLA Management (10)</v>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="20" t="n">
         <f>TestCoverage!F15</f>
-        <v>1</v>
-      </c>
-      <c r="C14" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="C14" s="20" t="n">
         <f>TestCoverage!G15</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D14" s="20" t="n">
         <f>TestCoverage!H15</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E14" s="20" t="n">
         <f>C14 + D14</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F14" s="19" t="n">
         <f>TestCoverage!B15</f>
-        <v>10</v>
-      </c>
-      <c r="G14" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="G14" s="18" t="n">
         <f>IF($F14=0,1,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="H14" s="19" t="str">
         <f>IF(G14=100%,"Not Automated","")</f>
@@ -4720,25 +4726,25 @@
         <f>TestCoverage!F16</f>
         <v/>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="20" t="n">
         <f>TestCoverage!G16</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="D15" s="20" t="n">
         <f>TestCoverage!H16</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E15" s="20" t="n">
         <f>C15 + D15</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F15" s="19" t="n">
         <f>TestCoverage!B16</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="18">
+        <v>0.0</v>
+      </c>
+      <c r="G15" s="18" t="n">
         <f>IF($F15=0,1,0)</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
       <c r="H15" s="19" t="str">
         <f>IF(G15=100%,"Not Automated","")</f>
@@ -4756,28 +4762,28 @@
     <row r="16" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="str">
         <f>TestCoverage!A17 &amp; " (" &amp; TestCoverage!B17 &amp; ")"</f>
-        <v>TOTAL (98)</v>
-      </c>
-      <c r="B16" s="20">
+        <v>TOTAL (104)</v>
+      </c>
+      <c r="B16" s="20" t="n">
         <f>TestCoverage!F17</f>
-        <v>0.96938775510204078</v>
-      </c>
-      <c r="C16" s="20">
+        <v>0.9519230769230769</v>
+      </c>
+      <c r="C16" s="20" t="n">
         <f>TestCoverage!G17</f>
-        <v>3.0612244897959183E-2</v>
-      </c>
-      <c r="D16" s="20">
+        <v>0.04807692307692308</v>
+      </c>
+      <c r="D16" s="20" t="n">
         <f>TestCoverage!H17</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="E16" s="20"/>
-      <c r="F16" s="19">
+      <c r="F16" s="19" t="n">
         <f>TestCoverage!B17</f>
-        <v>98</v>
-      </c>
-      <c r="G16" s="18">
+        <v>104.0</v>
+      </c>
+      <c r="G16" s="18" t="n">
         <f>COUNTIF(F2:F14,0)/COUNTA(A2:A14)</f>
-        <v>0.30769230769230771</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H16" s="19"/>
       <c r="I16" s="19"/>

</xml_diff>